<commit_message>
timer fix and indef remove
</commit_message>
<xml_diff>
--- a/data_project.xlsx
+++ b/data_project.xlsx
@@ -545,8 +545,8 @@
         <v>enum</v>
       </c>
       <c r="C11" t="str" xml:space="preserve">
-        <v xml:space="preserve">typedef enum {_x000d_
-    POSITION_LIGHTS, LOW_BEAMS_HEADLIGHTS, HIGH_BEAMS_HEADLIGHTS_x000d_
+        <v xml:space="preserve">typedef enum {
+    POSITION_LIGHTS, LOW_BEAMS_HEADLIGHTS, HIGH_BEAMS_HEADLIGHTS
 } light_type_t;</v>
       </c>
     </row>
@@ -558,8 +558,8 @@
         <v>enum</v>
       </c>
       <c r="C12" t="str" xml:space="preserve">
-        <v xml:space="preserve">typedef enum {_x000d_
-    RIGHT_BLINKERS, LEFT_BLINKERS, HAZARD_LIGHTS_x000d_
+        <v xml:space="preserve">typedef enum {
+    RIGHT_BLINKERS, LEFT_BLINKERS, HAZARD_LIGHTS
 } blinkers_type_t;</v>
       </c>
     </row>
@@ -571,8 +571,8 @@
         <v>enum</v>
       </c>
       <c r="C13" t="str" xml:space="preserve">
-        <v xml:space="preserve">typedef enum {_x000d_
-    NO_CHASSIS_PROBLEM = 0, TIRE_PRESSURE = 1, BRAKE_FAILURE = 2_x000d_
+        <v xml:space="preserve">typedef enum {
+    NO_CHASSIS_PROBLEM = 0, TIRE_PRESSURE = 1, BRAKE_FAILURE = 2
 } chassis_problems_type_t;</v>
       </c>
     </row>
@@ -584,8 +584,8 @@
         <v>enum</v>
       </c>
       <c r="C14" t="str" xml:space="preserve">
-        <v xml:space="preserve">typedef enum {_x000d_
-    NO_ENGINE_PROBLEM = 0, PRESSURE_DEFAULT = 1, COOLANT_TEMPERATURE = 2, OIL_OVERHEATING_x000d_
+        <v xml:space="preserve">typedef enum {
+    NO_ENGINE_PROBLEM = 0, PRESSURE_DEFAULT = 1, COOLANT_TEMPERATURE = 2, OIL_OVERHEATING
 } engine_problems_type_t;</v>
       </c>
     </row>
@@ -597,8 +597,8 @@
         <v>enum</v>
       </c>
       <c r="C15" t="str" xml:space="preserve">
-        <v xml:space="preserve">typedef enum {_x000d_
-    NO_BATTERY_PROBLEM = 0, DISCHARGED = 1, FAILURE = 2_x000d_
+        <v xml:space="preserve">typedef enum {
+    NO_BATTERY_PROBLEM = 0, DISCHARGED = 1, FAILURE = 2
 } battery_problems_type_t;</v>
       </c>
     </row>
@@ -610,8 +610,8 @@
         <v>enum</v>
       </c>
       <c r="C16" t="str" xml:space="preserve">
-        <v xml:space="preserve">typedef enum {_x000d_
-    POSITION_LIGHTS_ACTIVATION = 1, LOW_BEAMS_HEADLIGHTS_ACTIVATION = 2, HIGH_BEAMS_HEADLIGHTS_ACTIVATION = 3, RIGHT_BLINKERS_ACTIVATION = 4, LEFT_BLINKERS_ACTIVATION = 5_x000d_
+        <v xml:space="preserve">typedef enum {
+    POSITION_LIGHTS_ACTIVATION = 1, LOW_BEAMS_HEADLIGHTS_ACTIVATION = 2, HIGH_BEAMS_HEADLIGHTS_ACTIVATION = 3, RIGHT_BLINKERS_ACTIVATION = 4, LEFT_BLINKERS_ACTIVATION = 5
 } message_id_to_bgf_t;</v>
       </c>
     </row>
@@ -623,8 +623,8 @@
         <v>enum</v>
       </c>
       <c r="C17" t="str" xml:space="preserve">
-        <v xml:space="preserve">typedef enum {_x000d_
-    OFF=0, ON=1_x000d_
+        <v xml:space="preserve">typedef enum {
+    OFF=0, ON=1
 } state_lights_t;</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add the updated excel
</commit_message>
<xml_diff>
--- a/data_project.xlsx
+++ b/data_project.xlsx
@@ -447,7 +447,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="B4" t="str">
         <v>Atom</v>
@@ -863,7 +863,7 @@
         <v>timer_position_lights</v>
       </c>
       <c r="C16" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="E16" t="str">
         <v>0</v>
@@ -874,10 +874,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>timer_low_beams_lights</v>
+        <v>timer_low_beams_headlights</v>
       </c>
       <c r="C17" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="E17" t="str">
         <v>0</v>
@@ -888,10 +888,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>timer_high_beams_lights</v>
+        <v>timer_high_beams_headlights</v>
       </c>
       <c r="C18" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="E18" t="str">
         <v>0</v>
@@ -905,7 +905,7 @@
         <v>timer_right_blinkers</v>
       </c>
       <c r="C19" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="E19" t="str">
         <v>0</v>
@@ -919,7 +919,7 @@
         <v>timer_left_blinkers</v>
       </c>
       <c r="C20" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="E20" t="str">
         <v>0</v>
@@ -933,7 +933,7 @@
         <v>timer_hazard_lights</v>
       </c>
       <c r="C21" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="E21" t="str">
         <v>0</v>
@@ -947,7 +947,7 @@
         <v>timer_wipers</v>
       </c>
       <c r="C22" t="str">
-        <v>timer_t</v>
+        <v>timer_bcgv_t</v>
       </c>
       <c r="E22" t="str">
         <v>0</v>

</xml_diff>

<commit_message>
fix qu 8 + fix warnings + modify start.sh + put the variables declaration to the beginning of functions
</commit_message>
<xml_diff>
--- a/data_project.xlsx
+++ b/data_project.xlsx
@@ -491,9 +491,6 @@
       <c r="C7" t="str">
         <v>uint8_t</v>
       </c>
-      <c r="D7" t="str">
-        <v>[0;255]</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -532,9 +529,6 @@
       </c>
       <c r="C10" t="str">
         <v>uint8_t</v>
-      </c>
-      <c r="D10" t="str">
-        <v>[0;255]</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">

</xml_diff>